<commit_message>
Add Log Viewer & Fix Import
 - tambah log viewer mode development & local
 - perbaikan tampilan error gagal import
 - import berdasarkan nama battery
 - perubahan template excell
</commit_message>
<xml_diff>
--- a/public/template/excel/SampleImportVehicle.xlsx
+++ b/public/template/excel/SampleImportVehicle.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\x260\Documents\PEKERJAAN\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\x260\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9F4D5CB-737C-469E-8809-DE383C02BF43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2996CF5A-0244-47F2-852D-65DD61F13F02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{DCD433B4-E277-4D61-9B38-40B679A5AB11}"/>
   </bookViews>
@@ -45,82 +45,82 @@
     <t>VEHICLE</t>
   </si>
   <si>
-    <t>BATTERY</t>
-  </si>
-  <si>
-    <t>ALT 1</t>
-  </si>
-  <si>
-    <t>ALT 2</t>
-  </si>
-  <si>
-    <t>ALT 3</t>
-  </si>
-  <si>
     <t>YOUTUBE LINK</t>
   </si>
   <si>
     <t>HONDA HRV IVTECH</t>
   </si>
   <si>
-    <t xml:space="preserve">    Honda</t>
-  </si>
-  <si>
     <t>https://www.youtube.com/watch?v=yourvideolink</t>
   </si>
   <si>
     <t>TOYOTA CAMRY</t>
   </si>
   <si>
-    <t xml:space="preserve">      Toyota</t>
-  </si>
-  <si>
     <t>FORD FOCUS</t>
   </si>
   <si>
-    <t xml:space="preserve">        Ford</t>
-  </si>
-  <si>
     <t>NISSAN ALTIMA</t>
   </si>
   <si>
-    <t xml:space="preserve">      Nissan</t>
-  </si>
-  <si>
     <t>CHEVROLET CRUZE</t>
   </si>
   <si>
-    <t xml:space="preserve">    Chevrolet</t>
-  </si>
-  <si>
     <t>BMW X5</t>
   </si>
   <si>
-    <t xml:space="preserve">            BMW</t>
-  </si>
-  <si>
     <t>MERCEDES C-CLASS</t>
   </si>
   <si>
-    <t xml:space="preserve">  Mercedes</t>
-  </si>
-  <si>
     <t>AUDI A4</t>
   </si>
   <si>
-    <t xml:space="preserve">            Audi</t>
-  </si>
-  <si>
     <t>VOLKSWAGEN JETTA</t>
   </si>
   <si>
-    <t xml:space="preserve">  Volkswagen</t>
-  </si>
-  <si>
     <t>KIA SORENTO</t>
   </si>
   <si>
-    <t xml:space="preserve">        Kia</t>
+    <t>Honda</t>
+  </si>
+  <si>
+    <t>Toyota</t>
+  </si>
+  <si>
+    <t>Ford</t>
+  </si>
+  <si>
+    <t>Nissan</t>
+  </si>
+  <si>
+    <t>Chevrolet</t>
+  </si>
+  <si>
+    <t>BMW</t>
+  </si>
+  <si>
+    <t>Mercedes</t>
+  </si>
+  <si>
+    <t>Audi</t>
+  </si>
+  <si>
+    <t>Volkswagen</t>
+  </si>
+  <si>
+    <t>Kia</t>
+  </si>
+  <si>
+    <t>BATTERY NAME</t>
+  </si>
+  <si>
+    <t>BATTERY NAME ALTERNATE 3</t>
+  </si>
+  <si>
+    <t>BATTERY NAME ALTERNATE 2</t>
+  </si>
+  <si>
+    <t>BATTERY NAME ALTERNATE 4</t>
   </si>
 </sst>
 </file>
@@ -190,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -200,10 +200,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -223,7 +226,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -523,10 +526,9 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="7" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="26.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="47.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -580,169 +582,169 @@
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>3</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="5" t="s">
-        <v>10</v>
+        <v>4</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="6" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4" t="s">
-        <v>10</v>
+        <v>6</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4" t="s">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4" t="s">
-        <v>10</v>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4" t="s">
-        <v>10</v>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4" t="s">
-        <v>10</v>
+        <v>13</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4" t="s">
-        <v>10</v>
+        <v>14</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>